<commit_message>
Signed-in re-check of Axiom, GMGN, Pump.fun, FOMO (user logged in; quote-only)
Axiom: cross-chain Convert exists but amount clamps to wallet balance; deposit fees only at min.
GMGN: Convert needs 2FA + 3h lock. Pump.fun / GMGN deposits Solana-only. FOMO: unified balance, no quote.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bridg_Competitive_Benchmark.xlsx
+++ b/Bridg_Competitive_Benchmark.xlsx
@@ -2435,7 +2435,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED — bot protection + login required: axiom.trade serves a Cloudflare bot-verification page (HTTP 403) to a fresh browser; its official docs list no bridge/cross-chain transfer feature (only in-wallet Convert/swap and a Hyperliquid perps deposit), and any wallet features need an Axiom account.</t>
+          <t>BLOCKED — PARTIAL — no 100 USDC quote without funds. Signed-in check (user logged in; built-in browser, 2026-09-23): Axiom 'Exchange' has a cross-chain Convert (e.g. 'Swap USDC on Solana for USDC on Ethereum', indicative 1 USDC = 1.0000 USDC) but the amount field clamps to the wallet balance (0), so 100 can't be priced. Deposit auto-bridges EVM→Solana and shows fees only at its minimum: ETH→SOL USDC ($3 min) ~26s, impact −0.388%, fees ~$0.27 (gas $0.27, routing/liquidity &lt;$0.01); BSC→SOL ($2 min) ~26s, impact −8.357%, fees ~$0.21 (gas); Base→SOL ($2 min) ~26s, impact −0.455%, fees ~$0.02. Indicative only — not comparable to a 100 USDC quote.</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED — no bridge feature + login required: fomo.family abstracts chains behind a single USD balance (Solana/Base/BNB/Monad, 'no bridges needed'); no cross-chain USDC transfer quote exists, and deposit/withdraw/trade all require creating an account. Ethereum mainnet not supported.</t>
+          <t>BLOCKED — BLOCKED — signed-in check (user logged in): deposits accept USDC from Solana, Base, BNB Chain, Monad, Robinhood Chain, Arc, Ethereum into one USD cash balance; no fee/quote is shown at deposit and moving funds out needs a balance. No chain-to-chain quote.</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED — bot protection: gmgn.ai blocks a fresh browser with a Cloudflare 'you have been blocked' page (HTTP 403); official docs list no cross-chain bridge feature (only same-chain token swaps, which need a connected wallet/login).</t>
+          <t>BLOCKED — BLOCKED — signed-in check (user logged in): wallet menu has Convert, but it requires binding 2FA (a security-setting change the user must make) and then a 3-hour lock before Convert works. Deposit accepts SOL/USDT/USDC/USD1 on the Solana network only.</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>BLOCKED — Solana-only + login required: no general bridge; the only cross-chain feature is a MoonPay 'Cross Chain Deposit' into the user's own Pump.fun (Solana) account, which needs sign-in (and accepting the ToS modal). SOL-&gt;EVM directions are not offered at all.</t>
+          <t>BLOCKED — BLOCKED — signed-in check (user logged in): web Deposit is Solana-only ('Only send assets on the Solana network', min 0.01 SOL). No cross-chain quote on web; the MoonPay cross-chain deposit reported in news may be mobile-only.</t>
         </is>
       </c>
     </row>
@@ -52256,12 +52256,12 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>bot protection + login required: axiom.trade serves a Cloudflare bot-verification page (HTTP 403) to a fresh browser; its official docs list no bridge/cross-chain transfer feature (only in-wallet Convert/swap and a Hyperliquid perps deposit), and any wallet features need an Axiom account.</t>
+          <t>PARTIAL — no 100 USDC quote without funds. Signed-in check (user logged in; built-in browser, 2026-09-23): Axiom 'Exchange' has a cross-chain Convert (e.g. 'Swap USDC on Solana for USDC on Ethereum', indicative 1 USDC = 1.0000 USDC) but the amount field clamps to the wallet balance (0), so 100 can't be priced. Deposit auto-bridges EVM→Solana and shows fees only at its minimum: ETH→SOL USDC ($3 min) ~26s, impact −0.388%, fees ~$0.27 (gas $0.27, routing/liquidity &lt;$0.01); BSC→SOL ($2 min) ~26s, impact −8.357%, fees ~$0.21 (gas); Base→SOL ($2 min) ~26s, impact −0.455%, fees ~$0.02. Indicative only — not comparable to a 100 USDC quote.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T13:32:00Z</t>
+          <t>2026-09-23T14:07:33Z</t>
         </is>
       </c>
     </row>
@@ -52336,12 +52336,12 @@
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>no bridge feature + login required: fomo.family abstracts chains behind a single USD balance (Solana/Base/BNB/Monad, 'no bridges needed'); no cross-chain USDC transfer quote exists, and deposit/withdraw/trade all require creating an account. Ethereum mainnet not supported.</t>
+          <t>BLOCKED — signed-in check (user logged in): deposits accept USDC from Solana, Base, BNB Chain, Monad, Robinhood Chain, Arc, Ethereum into one USD cash balance; no fee/quote is shown at deposit and moving funds out needs a balance. No chain-to-chain quote.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T13:32:00Z</t>
+          <t>2026-09-23T14:07:33Z</t>
         </is>
       </c>
     </row>
@@ -52374,12 +52374,12 @@
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
-          <t>bot protection: gmgn.ai blocks a fresh browser with a Cloudflare 'you have been blocked' page (HTTP 403); official docs list no cross-chain bridge feature (only same-chain token swaps, which need a connected wallet/login).</t>
+          <t>BLOCKED — signed-in check (user logged in): wallet menu has Convert, but it requires binding 2FA (a security-setting change the user must make) and then a 3-hour lock before Convert works. Deposit accepts SOL/USDT/USDC/USD1 on the Solana network only.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T13:32:00Z</t>
+          <t>2026-09-23T14:07:33Z</t>
         </is>
       </c>
     </row>
@@ -52454,12 +52454,12 @@
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Solana-only + login required: no general bridge; the only cross-chain feature is a MoonPay 'Cross Chain Deposit' into the user's own Pump.fun (Solana) account, which needs sign-in (and accepting the ToS modal). SOL-&gt;EVM directions are not offered at all.</t>
+          <t>BLOCKED — signed-in check (user logged in): web Deposit is Solana-only ('Only send assets on the Solana network', min 0.01 SOL). No cross-chain quote on web; the MoonPay cross-chain deposit reported in news may be mobile-only.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23T13:32:00Z</t>
+          <t>2026-09-23T14:07:33Z</t>
         </is>
       </c>
     </row>
@@ -76172,7 +76172,7 @@
       </c>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>OpenSea swap (Relay; LI.FI on SOL→Base; 0% OpenSea fee promo) pays 11–13 bps less than Bridg's best on SOL→ETH, ETH→SOL and Base→SOL, and ~1 bp less on SOL→Base; OpenSea has no BNB Chain. Axiom and GMGN block automated browsers (Cloudflare 403) and document no bridge; FOMO has no chain-to-chain transfer ('no bridges needed'); Pump.fun only offers login-gated deposits into Solana.</t>
+          <t>OpenSea swap (Relay; LI.FI on SOL→Base; 0% OpenSea fee promo) pays 11–13 bps less than Bridg's best on SOL→ETH, ETH→SOL and Base→SOL, and ~1 bp less on SOL→Base; OpenSea has no BNB Chain. Signed in (by the user) and re-checked: Axiom has a cross-chain Convert and auto-bridged deposits, but Convert caps the amount at the wallet balance, so 100 USDC can't be priced unfunded (deposit fees shown only at its $2–3 minimum: ETH→SOL ~$0.27 gas, BSC→SOL ~$0.21, Base→SOL ~$0.02). GMGN's Convert needs 2FA plus a 3-hour lock; its deposits are Solana-only. Pump.fun's web deposit is Solana-only. FOMO pools deposits from 7 chains into one USD balance with no quote.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Explain gaps via Bridg API fee breakdowns (indicative, saved in data/api)
- Relay −20 bps into Solana = new USDC token-account cost (fresh recipient: +0.2009 USDC); matches relay.link otherwise
- Meson/Husher/Allbridge rows are flat fee formulas; LI.FI carries a 0.25 USDC 'LIFI Fixed Fee'
- CCTP gap = Circle forwarding fee Portal hides until wallet connect

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bridg_Competitive_Benchmark.xlsx
+++ b/Bridg_Competitive_Benchmark.xlsx
@@ -64697,17 +64697,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>serious</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C2" s="24" t="inlineStr">
         <is>
-          <t>Relay priced ~20 bps below relay.link on every EVM → Solana route</t>
+          <t>Relay ~20 bps below relay.link into Solana — explained: new USDC account cost</t>
         </is>
       </c>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>ETH→SOL, BSC→SOL, Base→SOL: −19.9 to −20.0 bps in every sample after adding back Bridg's 5 bps (~0.20 USDC more 'Relay fee'). SOL→ETH was −25 bps this campaign (Ethereum gas was elevated); SOL→BSC and SOL→Base match. Hypothesis (unverified): Bridg's quote includes Solana USDC token-account rent that relay.link omits when no recipient wallet is set.</t>
+          <t>ETH→SOL, BSC→SOL, Base→SOL: −19.9 to −20.0 bps in every sample after adding back Bridg's 5 bps. Verified via Bridg's API (indicative quotes, 14:45:35 UTC, saved in data/api/): for a recipient that already holds USDC, Bridg prices Relay at 99.945676 — identical to relay.link. For a fresh Solana address, Relay's 'destination fill gas' rises from 0.004 to 0.205 USDC (+20.1 bps): the cost of creating the recipient's USDC token account. Bridg's no-wallet page prices that case; relay.link's no-wallet page assumes the account exists. Mayan and NEAR Intents shift the same way. SOL→ETH was −25 bps this campaign (Ethereum gas elevated).</t>
         </is>
       </c>
     </row>
@@ -64727,7 +64727,7 @@
       </c>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>LI.FI: 15–96 bps below jumper.exchange's Best Return on every route. SimpleSwap: 48–272 bps below simpleswap.io's default floating 'Best rate'. Hypothesis (unverified): a different route/rate type or an integrator fee in Bridg's requests.</t>
+          <t>LI.FI: 15–96 bps below jumper.exchange's Best Return on every route. Bridg's API shows a 'LIFI Fixed Fee' of 0.25 USDC (25 bps) on its LI.FI row that Jumper doesn't charge, plus the ~0.20 new-account cost into Solana — together ~45 bps; the rest is unexplained (likely a different route). SimpleSwap: 48–272 bps below simpleswap.io's default floating 'Best rate'; Bridg's API lists no fee breakdown for it.</t>
         </is>
       </c>
     </row>
@@ -64742,12 +64742,12 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>Meson, Husher and Allbridge rows look like flat estimates, not live quotes</t>
+          <t>Meson and Husher rows are flat fee formulas, not live quotes (confirmed)</t>
         </is>
       </c>
       <c r="D4" s="23" t="inlineStr">
         <is>
-          <t>Bridg shows exactly 99.9 or 99.5 minus its own fee on every sample (99.85005 / 99.45025; 99.75015 on SOL→ETH where Bridg's fee tier was 15 bps). When Ethereum gas rose, Meson's own site dropped to 98.56 on SOL→ETH while Bridg still showed 99.75 (+134 bps). Husher's own site is 15–25 bps lower than Bridg's row. Allbridge matches only because its site also shows a flat 99.90.</t>
+          <t>Bridg's API fee breakdown: Meson = a fixed 'Meson LP fee' of 0.50 USDC; Husher = fixed 0.20 exchange fee + 0.30 delivery fee; Allbridge = fixed 0.10 CCTP service fee. So Bridg shows exactly 99.5/99.9 minus its own fee (99.45025 / 99.85005; 99.75015 on SOL→ETH at the 15 bps tier). When Ethereum gas rose, Meson's own site dropped to 98.56 on SOL→ETH while Bridg still showed 99.75 (+134 bps). Husher's own site charges 0.35% (not 0.20), so it's 15–25 bps lower than Bridg's row. Allbridge matches because its site also shows a flat 99.90.</t>
         </is>
       </c>
     </row>
@@ -64842,12 +64842,12 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>CCTP gap is a comparison limit, not a verdict</t>
+          <t>CCTP gap is Portal hiding a fee, not a Bridg error</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Circle's own bridge has no Solana, so CCTP is read from Portal (Wormhole), which hides its executor fee until a wallet connects. Portal's 99.99 is before that fee; Bridg's CCTP row (96.52 on SOL→ETH, −332 bps this campaign) likely includes Ethereum destination gas. Into Solana the gap is −14 to −15 bps.</t>
+          <t>Circle's own bridge has no Solana, so CCTP is read from Portal (Wormhole), which hides its relayer fee until a wallet connects. Bridg's API itemises it: 'Circle Forwarding Service fee and destination gas' = 0.16 USDC on ETH→SOL, which is the −14 to −15 bps gap into Solana. On SOL→ETH (−332 bps this campaign) the same line carries Ethereum destination gas, which was elevated.</t>
         </is>
       </c>
     </row>
@@ -65333,30 +65333,24 @@
     </row>
     <row r="26">
       <c r="A26" s="25">
-        <f>Issues!C2</f>
+        <f>Issues!C3</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25">
-        <f>Issues!C3</f>
+        <f>Issues!C4</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="25">
-        <f>Issues!C4</f>
+        <f>Issues!C5</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="25">
-        <f>Issues!C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="25">
         <f>Issues!C6</f>
         <v/>
       </c>
@@ -65369,10 +65363,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A33:G33"/>
     <mergeCell ref="A28:G28"/>

</xml_diff>

<commit_message>
Rename visible 'Bridg' to BRDG across dashboard, workbook, docs and pitch
Code identifiers and scraped page text (e.g. the 'Bridg fee' label) unchanged; pitch PDF now BRDG_x_OpenSea.pdf.
Fix dot plot negative width on very narrow viewports.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bridg_Competitive_Benchmark.xlsx
+++ b/Bridg_Competitive_Benchmark.xlsx
@@ -580,7 +580,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bridg Competitive Benchmark</t>
+          <t>BRDG Competitive Benchmark</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Routes where Bridg's best beat every direct quote</t>
+          <t>Routes where BRDG's best beat every direct quote</t>
         </is>
       </c>
       <c r="B5" s="5">
@@ -612,7 +612,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Venue pairs where Bridg's listing matches the venue's site</t>
+          <t>Venue pairs where BRDG's listing matches the venue's site</t>
         </is>
       </c>
       <c r="B6" s="5">
@@ -623,29 +623,29 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>… Bridg lists LESS than the venue's own site</t>
+          <t>… BRDG lists LESS than the venue's own site</t>
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Venue Analysis'!$Z$5:$Z$74,"Bridg LOWER*")</f>
+        <f>COUNTIF('Venue Analysis'!$Z$5:$Z$74,"BRDG LOWER*")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>… Bridg lists MORE than the venue's own site</t>
+          <t>… BRDG lists MORE than the venue's own site</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('Venue Analysis'!$Z$5:$Z$74,"Bridg HIGHER*")</f>
+        <f>COUNTIF('Venue Analysis'!$Z$5:$Z$74,"BRDG HIGHER*")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>… venue quotes on its site but is missing from Bridg</t>
+          <t>… venue quotes on its site but is missing from BRDG</t>
         </is>
       </c>
       <c r="B9" s="5">
@@ -656,7 +656,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Worst venue-accuracy gap (bps, ex-Bridg fee)</t>
+          <t>Worst venue-accuracy gap (bps, ex-BRDG fee)</t>
         </is>
       </c>
       <c r="B10" s="6">
@@ -714,7 +714,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Route winners (Bridg best vs best direct quote)</t>
+          <t>Route winners (BRDG best vs best direct quote)</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Bridg best</t>
+          <t>BRDG best</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Bridg vs best (bps)</t>
+          <t>BRDG vs best (bps)</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Sites Bridg beats</t>
+          <t>Sites BRDG beats</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Sites beating Bridg</t>
+          <t>Sites beating BRDG</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Venue accuracy (avg gap ex-Bridg fee, bps) — Bridg listed vs venue's own site</t>
+          <t>Venue accuracy (avg gap ex-BRDG fee, bps) — BRDG listed vs venue's own site</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Green = linked from other sheets. Red cells: Bridg lower / going direct pays more; blue: Bridg higher / Bridg pays more. Hypotheses in Issues are unverified.</t>
+          <t>Green = linked from other sheets. Red cells: BRDG lower / going direct pays more; blue: BRDG higher / BRDG pays more. Hypotheses in Issues are unverified.</t>
         </is>
       </c>
     </row>
@@ -2102,14 +2102,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Competitor Matrix — does a user get more on Bridg, or by going direct?</t>
+          <t>Competitor Matrix — does a user get more on BRDG, or by going direct?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Savings (bps) = (Bridg best − other) / 100 × 10,000. Positive = Bridg pays more. Bridg best = what Bridg's own page says you receive on its best-price route. Source-chain gas paid separately is not counted on either side.</t>
+          <t>Savings (bps) = (BRDG best − other) / 100 × 10,000. Positive = BRDG pays more. BRDG best = what BRDG's own page says you receive on its best-price route. Source-chain gas paid separately is not counted on either side.</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Bridg best (avg)</t>
+          <t>BRDG best (avg)</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -3205,17 +3205,17 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>Bridg vs best (bps)</t>
+          <t>BRDG vs best (bps)</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
-          <t>Sites Bridg beats</t>
+          <t>Sites BRDG beats</t>
         </is>
       </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>Sites beating Bridg</t>
+          <t>Sites beating BRDG</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="B28" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;ETH",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;ETH",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C28" s="17">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Bridg best is averaged per synchronized run (Raw Quotes); savings compare it with the best per-site average.</t>
+          <t>BRDG best is averaged per synchronized run (Raw Quotes); savings compare it with the best per-site average.</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="B29" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"ETH-&gt;SOL",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"ETH-&gt;SOL",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C29" s="17">
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="B30" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;BSC",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;BSC",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C30" s="17">
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="B31" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"BSC-&gt;SOL",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"BSC-&gt;SOL",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C31" s="17">
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="B32" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;Base",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"SOL-&gt;Base",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C32" s="17">
@@ -3386,7 +3386,7 @@
         </is>
       </c>
       <c r="B33" s="10">
-        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"Base-&gt;SOL",'Raw Quotes'!$D:$D,"Bridg",'Raw Quotes'!$F:$F,"OK"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Raw Quotes'!$K:$K,'Raw Quotes'!$B:$B,"Base-&gt;SOL",'Raw Quotes'!$D:$D,"BRDG",'Raw Quotes'!$F:$F,"OK"),"")</f>
         <v/>
       </c>
       <c r="C33" s="17">
@@ -3440,12 +3440,12 @@
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>Bridg best</t>
+          <t>BRDG best</t>
         </is>
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>Bridg best via</t>
+          <t>BRDG best via</t>
         </is>
       </c>
       <c r="G36" s="18" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="J36" s="18" t="inlineStr">
         <is>
-          <t>Bridg value read (UTC)</t>
+          <t>BRDG value read (UTC)</t>
         </is>
       </c>
       <c r="K36" s="18" t="inlineStr">
@@ -14425,14 +14425,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Venue Analysis — is Bridg's listed quote for each venue the same as the venue's own site?</t>
+          <t>Venue Analysis — is BRDG's listed quote for each venue the same as the venue's own site?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gap (bps) = (Bridg listed − venue direct) / 100 × 10,000. Ex-fee adds Bridg's platform fee back. Direct = venue out − any USDC fee charged on top of the 100 input. Blue = observed inputs; black = formulas.</t>
+          <t>Gap (bps) = (BRDG listed − venue direct) / 100 × 10,000. Ex-fee adds BRDG's platform fee back. Direct = venue out − any USDC fee charged on top of the 100 input. Blue = observed inputs; black = formulas.</t>
         </is>
       </c>
     </row>
@@ -14454,7 +14454,7 @@
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>Bridg listed</t>
+          <t>BRDG listed</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
       <c r="J4" s="18" t="inlineStr">
         <is>
-          <t>Bridg fee (USDC)</t>
+          <t>BRDG fee (USDC)</t>
         </is>
       </c>
       <c r="K4" s="18" t="inlineStr">
@@ -14504,7 +14504,7 @@
       </c>
       <c r="N4" s="18" t="inlineStr">
         <is>
-          <t>Bridg value read (UTC)</t>
+          <t>BRDG value read (UTC)</t>
         </is>
       </c>
       <c r="O4" s="18" t="inlineStr">
@@ -14529,12 +14529,12 @@
       </c>
       <c r="T4" s="18" t="inlineStr">
         <is>
-          <t>Listed on Bridg</t>
+          <t>Listed on BRDG</t>
         </is>
       </c>
       <c r="U4" s="18" t="inlineStr">
         <is>
-          <t>Bridg avg</t>
+          <t>BRDG avg</t>
         </is>
       </c>
       <c r="V4" s="18" t="inlineStr">
@@ -14652,7 +14652,7 @@
         <v>2</v>
       </c>
       <c r="Z5" s="4">
-        <f>IF(T5=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X5)),"No direct quote",IF(ABS(X5)&lt;=Y5,"Match (net of Bridg fee)",IF(ABS(W5)&lt;=Y5,"Match (Bridg fee not applied)",IF(X5&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T5=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X5)),"No direct quote",IF(ABS(X5)&lt;=Y5,"Match (net of BRDG fee)",IF(ABS(W5)&lt;=Y5,"Match (BRDG fee not applied)",IF(X5&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -14745,7 +14745,7 @@
         <v>2</v>
       </c>
       <c r="Z6" s="4">
-        <f>IF(T6=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X6)),"No direct quote",IF(ABS(X6)&lt;=Y6,"Match (net of Bridg fee)",IF(ABS(W6)&lt;=Y6,"Match (Bridg fee not applied)",IF(X6&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T6=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X6)),"No direct quote",IF(ABS(X6)&lt;=Y6,"Match (net of BRDG fee)",IF(ABS(W6)&lt;=Y6,"Match (BRDG fee not applied)",IF(X6&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -14838,7 +14838,7 @@
         <v>2</v>
       </c>
       <c r="Z7" s="4">
-        <f>IF(T7=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X7)),"No direct quote",IF(ABS(X7)&lt;=Y7,"Match (net of Bridg fee)",IF(ABS(W7)&lt;=Y7,"Match (Bridg fee not applied)",IF(X7&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T7=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X7)),"No direct quote",IF(ABS(X7)&lt;=Y7,"Match (net of BRDG fee)",IF(ABS(W7)&lt;=Y7,"Match (BRDG fee not applied)",IF(X7&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -14937,7 +14937,7 @@
         <v>2</v>
       </c>
       <c r="Z8" s="4">
-        <f>IF(T8=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X8)),"No direct quote",IF(ABS(X8)&lt;=Y8,"Match (net of Bridg fee)",IF(ABS(W8)&lt;=Y8,"Match (Bridg fee not applied)",IF(X8&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T8=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X8)),"No direct quote",IF(ABS(X8)&lt;=Y8,"Match (net of BRDG fee)",IF(ABS(W8)&lt;=Y8,"Match (BRDG fee not applied)",IF(X8&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15036,7 +15036,7 @@
         <v>4</v>
       </c>
       <c r="Z9" s="4">
-        <f>IF(T9=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X9)),"No direct quote",IF(ABS(X9)&lt;=Y9,"Match (net of Bridg fee)",IF(ABS(W9)&lt;=Y9,"Match (Bridg fee not applied)",IF(X9&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T9=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X9)),"No direct quote",IF(ABS(X9)&lt;=Y9,"Match (net of BRDG fee)",IF(ABS(W9)&lt;=Y9,"Match (BRDG fee not applied)",IF(X9&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15135,7 +15135,7 @@
         <v>2</v>
       </c>
       <c r="Z10" s="4">
-        <f>IF(T10=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X10)),"No direct quote",IF(ABS(X10)&lt;=Y10,"Match (net of Bridg fee)",IF(ABS(W10)&lt;=Y10,"Match (Bridg fee not applied)",IF(X10&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T10=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X10)),"No direct quote",IF(ABS(X10)&lt;=Y10,"Match (net of BRDG fee)",IF(ABS(W10)&lt;=Y10,"Match (BRDG fee not applied)",IF(X10&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15232,7 +15232,7 @@
         <v>2</v>
       </c>
       <c r="Z11" s="4">
-        <f>IF(T11=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X11)),"No direct quote",IF(ABS(X11)&lt;=Y11,"Match (net of Bridg fee)",IF(ABS(W11)&lt;=Y11,"Match (Bridg fee not applied)",IF(X11&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T11=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X11)),"No direct quote",IF(ABS(X11)&lt;=Y11,"Match (net of BRDG fee)",IF(ABS(W11)&lt;=Y11,"Match (BRDG fee not applied)",IF(X11&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
         <v>2</v>
       </c>
       <c r="Z12" s="4">
-        <f>IF(T12=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X12)),"No direct quote",IF(ABS(X12)&lt;=Y12,"Match (net of Bridg fee)",IF(ABS(W12)&lt;=Y12,"Match (Bridg fee not applied)",IF(X12&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T12=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X12)),"No direct quote",IF(ABS(X12)&lt;=Y12,"Match (net of BRDG fee)",IF(ABS(W12)&lt;=Y12,"Match (BRDG fee not applied)",IF(X12&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15426,7 +15426,7 @@
         <v>2</v>
       </c>
       <c r="Z13" s="4">
-        <f>IF(T13=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X13)),"No direct quote",IF(ABS(X13)&lt;=Y13,"Match (net of Bridg fee)",IF(ABS(W13)&lt;=Y13,"Match (Bridg fee not applied)",IF(X13&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T13=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X13)),"No direct quote",IF(ABS(X13)&lt;=Y13,"Match (net of BRDG fee)",IF(ABS(W13)&lt;=Y13,"Match (BRDG fee not applied)",IF(X13&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15519,7 +15519,7 @@
         <v>2</v>
       </c>
       <c r="Z14" s="4">
-        <f>IF(T14=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X14)),"No direct quote",IF(ABS(X14)&lt;=Y14,"Match (net of Bridg fee)",IF(ABS(W14)&lt;=Y14,"Match (Bridg fee not applied)",IF(X14&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T14=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X14)),"No direct quote",IF(ABS(X14)&lt;=Y14,"Match (net of BRDG fee)",IF(ABS(W14)&lt;=Y14,"Match (BRDG fee not applied)",IF(X14&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15612,7 +15612,7 @@
         <v>2</v>
       </c>
       <c r="Z15" s="4">
-        <f>IF(T15=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X15)),"No direct quote",IF(ABS(X15)&lt;=Y15,"Match (net of Bridg fee)",IF(ABS(W15)&lt;=Y15,"Match (Bridg fee not applied)",IF(X15&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T15=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X15)),"No direct quote",IF(ABS(X15)&lt;=Y15,"Match (net of BRDG fee)",IF(ABS(W15)&lt;=Y15,"Match (BRDG fee not applied)",IF(X15&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15705,7 +15705,7 @@
         <v>2</v>
       </c>
       <c r="Z16" s="4">
-        <f>IF(T16=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X16)),"No direct quote",IF(ABS(X16)&lt;=Y16,"Match (net of Bridg fee)",IF(ABS(W16)&lt;=Y16,"Match (Bridg fee not applied)",IF(X16&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T16=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X16)),"No direct quote",IF(ABS(X16)&lt;=Y16,"Match (net of BRDG fee)",IF(ABS(W16)&lt;=Y16,"Match (BRDG fee not applied)",IF(X16&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15806,7 +15806,7 @@
         <v>2</v>
       </c>
       <c r="Z17" s="4">
-        <f>IF(T17=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X17)),"No direct quote",IF(ABS(X17)&lt;=Y17,"Match (net of Bridg fee)",IF(ABS(W17)&lt;=Y17,"Match (Bridg fee not applied)",IF(X17&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T17=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X17)),"No direct quote",IF(ABS(X17)&lt;=Y17,"Match (net of BRDG fee)",IF(ABS(W17)&lt;=Y17,"Match (BRDG fee not applied)",IF(X17&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -15907,7 +15907,7 @@
         <v>2</v>
       </c>
       <c r="Z18" s="4">
-        <f>IF(T18=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X18)),"No direct quote",IF(ABS(X18)&lt;=Y18,"Match (net of Bridg fee)",IF(ABS(W18)&lt;=Y18,"Match (Bridg fee not applied)",IF(X18&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T18=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X18)),"No direct quote",IF(ABS(X18)&lt;=Y18,"Match (net of BRDG fee)",IF(ABS(W18)&lt;=Y18,"Match (BRDG fee not applied)",IF(X18&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16008,7 +16008,7 @@
         <v>2</v>
       </c>
       <c r="Z19" s="4">
-        <f>IF(T19=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X19)),"No direct quote",IF(ABS(X19)&lt;=Y19,"Match (net of Bridg fee)",IF(ABS(W19)&lt;=Y19,"Match (Bridg fee not applied)",IF(X19&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T19=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X19)),"No direct quote",IF(ABS(X19)&lt;=Y19,"Match (net of BRDG fee)",IF(ABS(W19)&lt;=Y19,"Match (BRDG fee not applied)",IF(X19&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16109,7 +16109,7 @@
         <v>2</v>
       </c>
       <c r="Z20" s="4">
-        <f>IF(T20=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X20)),"No direct quote",IF(ABS(X20)&lt;=Y20,"Match (net of Bridg fee)",IF(ABS(W20)&lt;=Y20,"Match (Bridg fee not applied)",IF(X20&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T20=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X20)),"No direct quote",IF(ABS(X20)&lt;=Y20,"Match (net of BRDG fee)",IF(ABS(W20)&lt;=Y20,"Match (BRDG fee not applied)",IF(X20&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16210,7 +16210,7 @@
         <v>2</v>
       </c>
       <c r="Z21" s="4">
-        <f>IF(T21=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X21)),"No direct quote",IF(ABS(X21)&lt;=Y21,"Match (net of Bridg fee)",IF(ABS(W21)&lt;=Y21,"Match (Bridg fee not applied)",IF(X21&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T21=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X21)),"No direct quote",IF(ABS(X21)&lt;=Y21,"Match (net of BRDG fee)",IF(ABS(W21)&lt;=Y21,"Match (BRDG fee not applied)",IF(X21&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16311,7 +16311,7 @@
         <v>4</v>
       </c>
       <c r="Z22" s="4">
-        <f>IF(T22=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X22)),"No direct quote",IF(ABS(X22)&lt;=Y22,"Match (net of Bridg fee)",IF(ABS(W22)&lt;=Y22,"Match (Bridg fee not applied)",IF(X22&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T22=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X22)),"No direct quote",IF(ABS(X22)&lt;=Y22,"Match (net of BRDG fee)",IF(ABS(W22)&lt;=Y22,"Match (BRDG fee not applied)",IF(X22&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16412,7 +16412,7 @@
         <v>2</v>
       </c>
       <c r="Z23" s="4">
-        <f>IF(T23=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X23)),"No direct quote",IF(ABS(X23)&lt;=Y23,"Match (net of Bridg fee)",IF(ABS(W23)&lt;=Y23,"Match (Bridg fee not applied)",IF(X23&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T23=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X23)),"No direct quote",IF(ABS(X23)&lt;=Y23,"Match (net of BRDG fee)",IF(ABS(W23)&lt;=Y23,"Match (BRDG fee not applied)",IF(X23&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16513,7 +16513,7 @@
         <v>2</v>
       </c>
       <c r="Z24" s="4">
-        <f>IF(T24=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X24)),"No direct quote",IF(ABS(X24)&lt;=Y24,"Match (net of Bridg fee)",IF(ABS(W24)&lt;=Y24,"Match (Bridg fee not applied)",IF(X24&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T24=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X24)),"No direct quote",IF(ABS(X24)&lt;=Y24,"Match (net of BRDG fee)",IF(ABS(W24)&lt;=Y24,"Match (BRDG fee not applied)",IF(X24&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16614,7 +16614,7 @@
         <v>2</v>
       </c>
       <c r="Z25" s="4">
-        <f>IF(T25=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X25)),"No direct quote",IF(ABS(X25)&lt;=Y25,"Match (net of Bridg fee)",IF(ABS(W25)&lt;=Y25,"Match (Bridg fee not applied)",IF(X25&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T25=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X25)),"No direct quote",IF(ABS(X25)&lt;=Y25,"Match (net of BRDG fee)",IF(ABS(W25)&lt;=Y25,"Match (BRDG fee not applied)",IF(X25&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16707,7 +16707,7 @@
         <v>2</v>
       </c>
       <c r="Z26" s="4">
-        <f>IF(T26=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X26)),"No direct quote",IF(ABS(X26)&lt;=Y26,"Match (net of Bridg fee)",IF(ABS(W26)&lt;=Y26,"Match (Bridg fee not applied)",IF(X26&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T26=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X26)),"No direct quote",IF(ABS(X26)&lt;=Y26,"Match (net of BRDG fee)",IF(ABS(W26)&lt;=Y26,"Match (BRDG fee not applied)",IF(X26&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16800,7 +16800,7 @@
         <v>2</v>
       </c>
       <c r="Z27" s="4">
-        <f>IF(T27=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X27)),"No direct quote",IF(ABS(X27)&lt;=Y27,"Match (net of Bridg fee)",IF(ABS(W27)&lt;=Y27,"Match (Bridg fee not applied)",IF(X27&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T27=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X27)),"No direct quote",IF(ABS(X27)&lt;=Y27,"Match (net of BRDG fee)",IF(ABS(W27)&lt;=Y27,"Match (BRDG fee not applied)",IF(X27&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16893,7 +16893,7 @@
         <v>2</v>
       </c>
       <c r="Z28" s="4">
-        <f>IF(T28=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X28)),"No direct quote",IF(ABS(X28)&lt;=Y28,"Match (net of Bridg fee)",IF(ABS(W28)&lt;=Y28,"Match (Bridg fee not applied)",IF(X28&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T28=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X28)),"No direct quote",IF(ABS(X28)&lt;=Y28,"Match (net of BRDG fee)",IF(ABS(W28)&lt;=Y28,"Match (BRDG fee not applied)",IF(X28&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -16986,7 +16986,7 @@
         <v>2</v>
       </c>
       <c r="Z29" s="4">
-        <f>IF(T29=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X29)),"No direct quote",IF(ABS(X29)&lt;=Y29,"Match (net of Bridg fee)",IF(ABS(W29)&lt;=Y29,"Match (Bridg fee not applied)",IF(X29&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T29=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X29)),"No direct quote",IF(ABS(X29)&lt;=Y29,"Match (net of BRDG fee)",IF(ABS(W29)&lt;=Y29,"Match (BRDG fee not applied)",IF(X29&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17079,7 +17079,7 @@
         <v>2</v>
       </c>
       <c r="Z30" s="4">
-        <f>IF(T30=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X30)),"No direct quote",IF(ABS(X30)&lt;=Y30,"Match (net of Bridg fee)",IF(ABS(W30)&lt;=Y30,"Match (Bridg fee not applied)",IF(X30&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T30=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X30)),"No direct quote",IF(ABS(X30)&lt;=Y30,"Match (net of BRDG fee)",IF(ABS(W30)&lt;=Y30,"Match (BRDG fee not applied)",IF(X30&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17172,7 +17172,7 @@
         <v>2</v>
       </c>
       <c r="Z31" s="4">
-        <f>IF(T31=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X31)),"No direct quote",IF(ABS(X31)&lt;=Y31,"Match (net of Bridg fee)",IF(ABS(W31)&lt;=Y31,"Match (Bridg fee not applied)",IF(X31&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T31=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X31)),"No direct quote",IF(ABS(X31)&lt;=Y31,"Match (net of BRDG fee)",IF(ABS(W31)&lt;=Y31,"Match (BRDG fee not applied)",IF(X31&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17269,7 +17269,7 @@
         <v>2</v>
       </c>
       <c r="Z32" s="4">
-        <f>IF(T32=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X32)),"No direct quote",IF(ABS(X32)&lt;=Y32,"Match (net of Bridg fee)",IF(ABS(W32)&lt;=Y32,"Match (Bridg fee not applied)",IF(X32&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T32=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X32)),"No direct quote",IF(ABS(X32)&lt;=Y32,"Match (net of BRDG fee)",IF(ABS(W32)&lt;=Y32,"Match (BRDG fee not applied)",IF(X32&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17366,7 +17366,7 @@
         <v>2</v>
       </c>
       <c r="Z33" s="4">
-        <f>IF(T33=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X33)),"No direct quote",IF(ABS(X33)&lt;=Y33,"Match (net of Bridg fee)",IF(ABS(W33)&lt;=Y33,"Match (Bridg fee not applied)",IF(X33&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T33=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X33)),"No direct quote",IF(ABS(X33)&lt;=Y33,"Match (net of BRDG fee)",IF(ABS(W33)&lt;=Y33,"Match (BRDG fee not applied)",IF(X33&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17463,7 +17463,7 @@
         <v>2</v>
       </c>
       <c r="Z34" s="4">
-        <f>IF(T34=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X34)),"No direct quote",IF(ABS(X34)&lt;=Y34,"Match (net of Bridg fee)",IF(ABS(W34)&lt;=Y34,"Match (Bridg fee not applied)",IF(X34&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T34=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X34)),"No direct quote",IF(ABS(X34)&lt;=Y34,"Match (net of BRDG fee)",IF(ABS(W34)&lt;=Y34,"Match (BRDG fee not applied)",IF(X34&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17560,7 +17560,7 @@
         <v>4</v>
       </c>
       <c r="Z35" s="4">
-        <f>IF(T35=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X35)),"No direct quote",IF(ABS(X35)&lt;=Y35,"Match (net of Bridg fee)",IF(ABS(W35)&lt;=Y35,"Match (Bridg fee not applied)",IF(X35&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T35=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X35)),"No direct quote",IF(ABS(X35)&lt;=Y35,"Match (net of BRDG fee)",IF(ABS(W35)&lt;=Y35,"Match (BRDG fee not applied)",IF(X35&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17657,7 +17657,7 @@
         <v>2</v>
       </c>
       <c r="Z36" s="4">
-        <f>IF(T36=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X36)),"No direct quote",IF(ABS(X36)&lt;=Y36,"Match (net of Bridg fee)",IF(ABS(W36)&lt;=Y36,"Match (Bridg fee not applied)",IF(X36&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T36=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X36)),"No direct quote",IF(ABS(X36)&lt;=Y36,"Match (net of BRDG fee)",IF(ABS(W36)&lt;=Y36,"Match (BRDG fee not applied)",IF(X36&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17754,7 +17754,7 @@
         <v>2</v>
       </c>
       <c r="Z37" s="4">
-        <f>IF(T37=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X37)),"No direct quote",IF(ABS(X37)&lt;=Y37,"Match (net of Bridg fee)",IF(ABS(W37)&lt;=Y37,"Match (Bridg fee not applied)",IF(X37&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T37=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X37)),"No direct quote",IF(ABS(X37)&lt;=Y37,"Match (net of BRDG fee)",IF(ABS(W37)&lt;=Y37,"Match (BRDG fee not applied)",IF(X37&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17847,7 +17847,7 @@
         <v>2</v>
       </c>
       <c r="Z38" s="4">
-        <f>IF(T38=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X38)),"No direct quote",IF(ABS(X38)&lt;=Y38,"Match (net of Bridg fee)",IF(ABS(W38)&lt;=Y38,"Match (Bridg fee not applied)",IF(X38&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T38=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X38)),"No direct quote",IF(ABS(X38)&lt;=Y38,"Match (net of BRDG fee)",IF(ABS(W38)&lt;=Y38,"Match (BRDG fee not applied)",IF(X38&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -17940,7 +17940,7 @@
         <v>2</v>
       </c>
       <c r="Z39" s="4">
-        <f>IF(T39=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X39)),"No direct quote",IF(ABS(X39)&lt;=Y39,"Match (net of Bridg fee)",IF(ABS(W39)&lt;=Y39,"Match (Bridg fee not applied)",IF(X39&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T39=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X39)),"No direct quote",IF(ABS(X39)&lt;=Y39,"Match (net of BRDG fee)",IF(ABS(W39)&lt;=Y39,"Match (BRDG fee not applied)",IF(X39&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18033,7 +18033,7 @@
         <v>2</v>
       </c>
       <c r="Z40" s="4">
-        <f>IF(T40=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X40)),"No direct quote",IF(ABS(X40)&lt;=Y40,"Match (net of Bridg fee)",IF(ABS(W40)&lt;=Y40,"Match (Bridg fee not applied)",IF(X40&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T40=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X40)),"No direct quote",IF(ABS(X40)&lt;=Y40,"Match (net of BRDG fee)",IF(ABS(W40)&lt;=Y40,"Match (BRDG fee not applied)",IF(X40&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18126,7 +18126,7 @@
         <v>2</v>
       </c>
       <c r="Z41" s="4">
-        <f>IF(T41=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X41)),"No direct quote",IF(ABS(X41)&lt;=Y41,"Match (net of Bridg fee)",IF(ABS(W41)&lt;=Y41,"Match (Bridg fee not applied)",IF(X41&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T41=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X41)),"No direct quote",IF(ABS(X41)&lt;=Y41,"Match (net of BRDG fee)",IF(ABS(W41)&lt;=Y41,"Match (BRDG fee not applied)",IF(X41&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18219,7 +18219,7 @@
         <v>2</v>
       </c>
       <c r="Z42" s="4">
-        <f>IF(T42=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X42)),"No direct quote",IF(ABS(X42)&lt;=Y42,"Match (net of Bridg fee)",IF(ABS(W42)&lt;=Y42,"Match (Bridg fee not applied)",IF(X42&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T42=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X42)),"No direct quote",IF(ABS(X42)&lt;=Y42,"Match (net of BRDG fee)",IF(ABS(W42)&lt;=Y42,"Match (BRDG fee not applied)",IF(X42&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18312,7 +18312,7 @@
         <v>2</v>
       </c>
       <c r="Z43" s="4">
-        <f>IF(T43=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X43)),"No direct quote",IF(ABS(X43)&lt;=Y43,"Match (net of Bridg fee)",IF(ABS(W43)&lt;=Y43,"Match (Bridg fee not applied)",IF(X43&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T43=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X43)),"No direct quote",IF(ABS(X43)&lt;=Y43,"Match (net of BRDG fee)",IF(ABS(W43)&lt;=Y43,"Match (BRDG fee not applied)",IF(X43&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18405,7 +18405,7 @@
         <v>4</v>
       </c>
       <c r="Z44" s="4">
-        <f>IF(T44=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X44)),"No direct quote",IF(ABS(X44)&lt;=Y44,"Match (net of Bridg fee)",IF(ABS(W44)&lt;=Y44,"Match (Bridg fee not applied)",IF(X44&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T44=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X44)),"No direct quote",IF(ABS(X44)&lt;=Y44,"Match (net of BRDG fee)",IF(ABS(W44)&lt;=Y44,"Match (BRDG fee not applied)",IF(X44&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18498,7 +18498,7 @@
         <v>2</v>
       </c>
       <c r="Z45" s="4">
-        <f>IF(T45=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X45)),"No direct quote",IF(ABS(X45)&lt;=Y45,"Match (net of Bridg fee)",IF(ABS(W45)&lt;=Y45,"Match (Bridg fee not applied)",IF(X45&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T45=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X45)),"No direct quote",IF(ABS(X45)&lt;=Y45,"Match (net of BRDG fee)",IF(ABS(W45)&lt;=Y45,"Match (BRDG fee not applied)",IF(X45&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18591,7 +18591,7 @@
         <v>2</v>
       </c>
       <c r="Z46" s="4">
-        <f>IF(T46=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X46)),"No direct quote",IF(ABS(X46)&lt;=Y46,"Match (net of Bridg fee)",IF(ABS(W46)&lt;=Y46,"Match (Bridg fee not applied)",IF(X46&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T46=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X46)),"No direct quote",IF(ABS(X46)&lt;=Y46,"Match (net of BRDG fee)",IF(ABS(W46)&lt;=Y46,"Match (BRDG fee not applied)",IF(X46&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18690,7 +18690,7 @@
         <v>2</v>
       </c>
       <c r="Z47" s="4">
-        <f>IF(T47=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X47)),"No direct quote",IF(ABS(X47)&lt;=Y47,"Match (net of Bridg fee)",IF(ABS(W47)&lt;=Y47,"Match (Bridg fee not applied)",IF(X47&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T47=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X47)),"No direct quote",IF(ABS(X47)&lt;=Y47,"Match (net of BRDG fee)",IF(ABS(W47)&lt;=Y47,"Match (BRDG fee not applied)",IF(X47&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18789,7 +18789,7 @@
         <v>2</v>
       </c>
       <c r="Z48" s="4">
-        <f>IF(T48=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X48)),"No direct quote",IF(ABS(X48)&lt;=Y48,"Match (net of Bridg fee)",IF(ABS(W48)&lt;=Y48,"Match (Bridg fee not applied)",IF(X48&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T48=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X48)),"No direct quote",IF(ABS(X48)&lt;=Y48,"Match (net of BRDG fee)",IF(ABS(W48)&lt;=Y48,"Match (BRDG fee not applied)",IF(X48&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18888,7 +18888,7 @@
         <v>2</v>
       </c>
       <c r="Z49" s="4">
-        <f>IF(T49=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X49)),"No direct quote",IF(ABS(X49)&lt;=Y49,"Match (net of Bridg fee)",IF(ABS(W49)&lt;=Y49,"Match (Bridg fee not applied)",IF(X49&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T49=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X49)),"No direct quote",IF(ABS(X49)&lt;=Y49,"Match (net of BRDG fee)",IF(ABS(W49)&lt;=Y49,"Match (BRDG fee not applied)",IF(X49&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -18985,7 +18985,7 @@
         <v>2</v>
       </c>
       <c r="Z50" s="4">
-        <f>IF(T50=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X50)),"No direct quote",IF(ABS(X50)&lt;=Y50,"Match (net of Bridg fee)",IF(ABS(W50)&lt;=Y50,"Match (Bridg fee not applied)",IF(X50&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T50=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X50)),"No direct quote",IF(ABS(X50)&lt;=Y50,"Match (net of BRDG fee)",IF(ABS(W50)&lt;=Y50,"Match (BRDG fee not applied)",IF(X50&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19082,7 +19082,7 @@
         <v>2</v>
       </c>
       <c r="Z51" s="4">
-        <f>IF(T51=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X51)),"No direct quote",IF(ABS(X51)&lt;=Y51,"Match (net of Bridg fee)",IF(ABS(W51)&lt;=Y51,"Match (Bridg fee not applied)",IF(X51&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T51=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X51)),"No direct quote",IF(ABS(X51)&lt;=Y51,"Match (net of BRDG fee)",IF(ABS(W51)&lt;=Y51,"Match (BRDG fee not applied)",IF(X51&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19179,7 +19179,7 @@
         <v>2</v>
       </c>
       <c r="Z52" s="4">
-        <f>IF(T52=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X52)),"No direct quote",IF(ABS(X52)&lt;=Y52,"Match (net of Bridg fee)",IF(ABS(W52)&lt;=Y52,"Match (Bridg fee not applied)",IF(X52&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T52=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X52)),"No direct quote",IF(ABS(X52)&lt;=Y52,"Match (net of BRDG fee)",IF(ABS(W52)&lt;=Y52,"Match (BRDG fee not applied)",IF(X52&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19274,7 +19274,7 @@
         <v>2</v>
       </c>
       <c r="Z53" s="4">
-        <f>IF(T53=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X53)),"No direct quote",IF(ABS(X53)&lt;=Y53,"Match (net of Bridg fee)",IF(ABS(W53)&lt;=Y53,"Match (Bridg fee not applied)",IF(X53&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T53=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X53)),"No direct quote",IF(ABS(X53)&lt;=Y53,"Match (net of BRDG fee)",IF(ABS(W53)&lt;=Y53,"Match (BRDG fee not applied)",IF(X53&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19369,7 +19369,7 @@
         <v>4</v>
       </c>
       <c r="Z54" s="4">
-        <f>IF(T54=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X54)),"No direct quote",IF(ABS(X54)&lt;=Y54,"Match (net of Bridg fee)",IF(ABS(W54)&lt;=Y54,"Match (Bridg fee not applied)",IF(X54&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T54=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X54)),"No direct quote",IF(ABS(X54)&lt;=Y54,"Match (net of BRDG fee)",IF(ABS(W54)&lt;=Y54,"Match (BRDG fee not applied)",IF(X54&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19464,7 +19464,7 @@
         <v>2</v>
       </c>
       <c r="Z55" s="4">
-        <f>IF(T55=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X55)),"No direct quote",IF(ABS(X55)&lt;=Y55,"Match (net of Bridg fee)",IF(ABS(W55)&lt;=Y55,"Match (Bridg fee not applied)",IF(X55&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T55=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X55)),"No direct quote",IF(ABS(X55)&lt;=Y55,"Match (net of BRDG fee)",IF(ABS(W55)&lt;=Y55,"Match (BRDG fee not applied)",IF(X55&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19561,7 +19561,7 @@
         <v>2</v>
       </c>
       <c r="Z56" s="4">
-        <f>IF(T56=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X56)),"No direct quote",IF(ABS(X56)&lt;=Y56,"Match (net of Bridg fee)",IF(ABS(W56)&lt;=Y56,"Match (Bridg fee not applied)",IF(X56&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T56=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X56)),"No direct quote",IF(ABS(X56)&lt;=Y56,"Match (net of BRDG fee)",IF(ABS(W56)&lt;=Y56,"Match (BRDG fee not applied)",IF(X56&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19658,7 +19658,7 @@
         <v>2</v>
       </c>
       <c r="Z57" s="4">
-        <f>IF(T57=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X57)),"No direct quote",IF(ABS(X57)&lt;=Y57,"Match (net of Bridg fee)",IF(ABS(W57)&lt;=Y57,"Match (Bridg fee not applied)",IF(X57&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T57=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X57)),"No direct quote",IF(ABS(X57)&lt;=Y57,"Match (net of BRDG fee)",IF(ABS(W57)&lt;=Y57,"Match (BRDG fee not applied)",IF(X57&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19755,7 +19755,7 @@
         <v>2</v>
       </c>
       <c r="Z58" s="4">
-        <f>IF(T58=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X58)),"No direct quote",IF(ABS(X58)&lt;=Y58,"Match (net of Bridg fee)",IF(ABS(W58)&lt;=Y58,"Match (Bridg fee not applied)",IF(X58&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T58=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X58)),"No direct quote",IF(ABS(X58)&lt;=Y58,"Match (net of BRDG fee)",IF(ABS(W58)&lt;=Y58,"Match (BRDG fee not applied)",IF(X58&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19852,7 +19852,7 @@
         <v>2</v>
       </c>
       <c r="Z59" s="4">
-        <f>IF(T59=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X59)),"No direct quote",IF(ABS(X59)&lt;=Y59,"Match (net of Bridg fee)",IF(ABS(W59)&lt;=Y59,"Match (Bridg fee not applied)",IF(X59&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T59=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X59)),"No direct quote",IF(ABS(X59)&lt;=Y59,"Match (net of BRDG fee)",IF(ABS(W59)&lt;=Y59,"Match (BRDG fee not applied)",IF(X59&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -19949,7 +19949,7 @@
         <v>2</v>
       </c>
       <c r="Z60" s="4">
-        <f>IF(T60=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X60)),"No direct quote",IF(ABS(X60)&lt;=Y60,"Match (net of Bridg fee)",IF(ABS(W60)&lt;=Y60,"Match (Bridg fee not applied)",IF(X60&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T60=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X60)),"No direct quote",IF(ABS(X60)&lt;=Y60,"Match (net of BRDG fee)",IF(ABS(W60)&lt;=Y60,"Match (BRDG fee not applied)",IF(X60&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20046,7 +20046,7 @@
         <v>2</v>
       </c>
       <c r="Z61" s="4">
-        <f>IF(T61=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X61)),"No direct quote",IF(ABS(X61)&lt;=Y61,"Match (net of Bridg fee)",IF(ABS(W61)&lt;=Y61,"Match (Bridg fee not applied)",IF(X61&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T61=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X61)),"No direct quote",IF(ABS(X61)&lt;=Y61,"Match (net of BRDG fee)",IF(ABS(W61)&lt;=Y61,"Match (BRDG fee not applied)",IF(X61&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20143,7 +20143,7 @@
         <v>2</v>
       </c>
       <c r="Z62" s="4">
-        <f>IF(T62=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X62)),"No direct quote",IF(ABS(X62)&lt;=Y62,"Match (net of Bridg fee)",IF(ABS(W62)&lt;=Y62,"Match (Bridg fee not applied)",IF(X62&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T62=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X62)),"No direct quote",IF(ABS(X62)&lt;=Y62,"Match (net of BRDG fee)",IF(ABS(W62)&lt;=Y62,"Match (BRDG fee not applied)",IF(X62&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20240,7 +20240,7 @@
         <v>2</v>
       </c>
       <c r="Z63" s="4">
-        <f>IF(T63=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X63)),"No direct quote",IF(ABS(X63)&lt;=Y63,"Match (net of Bridg fee)",IF(ABS(W63)&lt;=Y63,"Match (Bridg fee not applied)",IF(X63&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T63=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X63)),"No direct quote",IF(ABS(X63)&lt;=Y63,"Match (net of BRDG fee)",IF(ABS(W63)&lt;=Y63,"Match (BRDG fee not applied)",IF(X63&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20337,7 +20337,7 @@
         <v>2</v>
       </c>
       <c r="Z64" s="4">
-        <f>IF(T64=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X64)),"No direct quote",IF(ABS(X64)&lt;=Y64,"Match (net of Bridg fee)",IF(ABS(W64)&lt;=Y64,"Match (Bridg fee not applied)",IF(X64&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T64=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X64)),"No direct quote",IF(ABS(X64)&lt;=Y64,"Match (net of BRDG fee)",IF(ABS(W64)&lt;=Y64,"Match (BRDG fee not applied)",IF(X64&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20430,7 +20430,7 @@
         <v>2</v>
       </c>
       <c r="Z65" s="4">
-        <f>IF(T65=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X65)),"No direct quote",IF(ABS(X65)&lt;=Y65,"Match (net of Bridg fee)",IF(ABS(W65)&lt;=Y65,"Match (Bridg fee not applied)",IF(X65&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T65=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X65)),"No direct quote",IF(ABS(X65)&lt;=Y65,"Match (net of BRDG fee)",IF(ABS(W65)&lt;=Y65,"Match (BRDG fee not applied)",IF(X65&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20523,7 +20523,7 @@
         <v>4</v>
       </c>
       <c r="Z66" s="4">
-        <f>IF(T66=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X66)),"No direct quote",IF(ABS(X66)&lt;=Y66,"Match (net of Bridg fee)",IF(ABS(W66)&lt;=Y66,"Match (Bridg fee not applied)",IF(X66&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T66=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X66)),"No direct quote",IF(ABS(X66)&lt;=Y66,"Match (net of BRDG fee)",IF(ABS(W66)&lt;=Y66,"Match (BRDG fee not applied)",IF(X66&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20616,7 +20616,7 @@
         <v>2</v>
       </c>
       <c r="Z67" s="4">
-        <f>IF(T67=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X67)),"No direct quote",IF(ABS(X67)&lt;=Y67,"Match (net of Bridg fee)",IF(ABS(W67)&lt;=Y67,"Match (Bridg fee not applied)",IF(X67&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T67=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X67)),"No direct quote",IF(ABS(X67)&lt;=Y67,"Match (net of BRDG fee)",IF(ABS(W67)&lt;=Y67,"Match (BRDG fee not applied)",IF(X67&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20709,7 +20709,7 @@
         <v>2</v>
       </c>
       <c r="Z68" s="4">
-        <f>IF(T68=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X68)),"No direct quote",IF(ABS(X68)&lt;=Y68,"Match (net of Bridg fee)",IF(ABS(W68)&lt;=Y68,"Match (Bridg fee not applied)",IF(X68&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T68=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X68)),"No direct quote",IF(ABS(X68)&lt;=Y68,"Match (net of BRDG fee)",IF(ABS(W68)&lt;=Y68,"Match (BRDG fee not applied)",IF(X68&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20802,7 +20802,7 @@
         <v>2</v>
       </c>
       <c r="Z69" s="4">
-        <f>IF(T69=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X69)),"No direct quote",IF(ABS(X69)&lt;=Y69,"Match (net of Bridg fee)",IF(ABS(W69)&lt;=Y69,"Match (Bridg fee not applied)",IF(X69&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T69=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X69)),"No direct quote",IF(ABS(X69)&lt;=Y69,"Match (net of BRDG fee)",IF(ABS(W69)&lt;=Y69,"Match (BRDG fee not applied)",IF(X69&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20895,7 +20895,7 @@
         <v>2</v>
       </c>
       <c r="Z70" s="4">
-        <f>IF(T70=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X70)),"No direct quote",IF(ABS(X70)&lt;=Y70,"Match (net of Bridg fee)",IF(ABS(W70)&lt;=Y70,"Match (Bridg fee not applied)",IF(X70&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T70=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X70)),"No direct quote",IF(ABS(X70)&lt;=Y70,"Match (net of BRDG fee)",IF(ABS(W70)&lt;=Y70,"Match (BRDG fee not applied)",IF(X70&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -20988,7 +20988,7 @@
         <v>2</v>
       </c>
       <c r="Z71" s="4">
-        <f>IF(T71=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X71)),"No direct quote",IF(ABS(X71)&lt;=Y71,"Match (net of Bridg fee)",IF(ABS(W71)&lt;=Y71,"Match (Bridg fee not applied)",IF(X71&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T71=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X71)),"No direct quote",IF(ABS(X71)&lt;=Y71,"Match (net of BRDG fee)",IF(ABS(W71)&lt;=Y71,"Match (BRDG fee not applied)",IF(X71&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -21081,7 +21081,7 @@
         <v>2</v>
       </c>
       <c r="Z72" s="4">
-        <f>IF(T72=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X72)),"No direct quote",IF(ABS(X72)&lt;=Y72,"Match (net of Bridg fee)",IF(ABS(W72)&lt;=Y72,"Match (Bridg fee not applied)",IF(X72&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T72=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X72)),"No direct quote",IF(ABS(X72)&lt;=Y72,"Match (net of BRDG fee)",IF(ABS(W72)&lt;=Y72,"Match (BRDG fee not applied)",IF(X72&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -21174,7 +21174,7 @@
         <v>2</v>
       </c>
       <c r="Z73" s="4">
-        <f>IF(T73=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X73)),"No direct quote",IF(ABS(X73)&lt;=Y73,"Match (net of Bridg fee)",IF(ABS(W73)&lt;=Y73,"Match (Bridg fee not applied)",IF(X73&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T73=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X73)),"No direct quote",IF(ABS(X73)&lt;=Y73,"Match (net of BRDG fee)",IF(ABS(W73)&lt;=Y73,"Match (BRDG fee not applied)",IF(X73&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -21271,7 +21271,7 @@
         <v>2</v>
       </c>
       <c r="Z74" s="4">
-        <f>IF(T74=0,"NOT LISTED on Bridg",IF(NOT(ISNUMBER(X74)),"No direct quote",IF(ABS(X74)&lt;=Y74,"Match (net of Bridg fee)",IF(ABS(W74)&lt;=Y74,"Match (Bridg fee not applied)",IF(X74&lt;0,"Bridg LOWER than venue","Bridg HIGHER than venue")))))</f>
+        <f>IF(T74=0,"NOT LISTED on BRDG",IF(NOT(ISNUMBER(X74)),"No direct quote",IF(ABS(X74)&lt;=Y74,"Match (net of BRDG fee)",IF(ABS(W74)&lt;=Y74,"Match (BRDG fee not applied)",IF(X74&lt;0,"BRDG LOWER than venue","BRDG HIGHER than venue")))))</f>
         <v/>
       </c>
     </row>
@@ -28997,7 +28997,7 @@
       </c>
       <c r="G1" s="18" t="inlineStr">
         <is>
-          <t>Δ vs Bridg (s)</t>
+          <t>Δ vs BRDG (s)</t>
         </is>
       </c>
       <c r="H1" s="18" t="inlineStr">
@@ -29042,7 +29042,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -29955,7 +29955,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -30868,7 +30868,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -31781,7 +31781,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -32694,7 +32694,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -33546,7 +33546,7 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -34459,7 +34459,7 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -35067,7 +35067,7 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -35675,7 +35675,7 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -36222,7 +36222,7 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -36891,7 +36891,7 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -37560,7 +37560,7 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
@@ -38229,7 +38229,7 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
@@ -39081,7 +39081,7 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
@@ -39933,7 +39933,7 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
@@ -40785,7 +40785,7 @@
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
@@ -41698,7 +41698,7 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
@@ -42611,7 +42611,7 @@
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
@@ -44039,7 +44039,7 @@
       </c>
       <c r="E1" s="18" t="inlineStr">
         <is>
-          <t>Bridg venue id</t>
+          <t>BRDG venue id</t>
         </is>
       </c>
       <c r="F1" s="18" t="inlineStr">
@@ -44061,7 +44061,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -44878,7 +44878,7 @@
       </c>
       <c r="J1" s="18" t="inlineStr">
         <is>
-          <t>Δ read vs Bridg (s)</t>
+          <t>Δ read vs BRDG (s)</t>
         </is>
       </c>
       <c r="K1" s="18" t="inlineStr">
@@ -44943,7 +44943,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -46180,7 +46180,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -47417,7 +47417,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -48235,7 +48235,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -49136,7 +49136,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -50290,7 +50290,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -51527,7 +51527,7 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -52758,7 +52758,7 @@
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
@@ -53979,7 +53979,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -54797,7 +54797,7 @@
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
@@ -55698,7 +55698,7 @@
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E133" s="4" t="inlineStr">
@@ -56852,7 +56852,7 @@
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E147" s="4" t="inlineStr">
@@ -58089,7 +58089,7 @@
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
@@ -59326,7 +59326,7 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
@@ -60563,7 +60563,7 @@
       </c>
       <c r="D192" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E192" s="4" t="inlineStr">
@@ -61365,7 +61365,7 @@
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr">
@@ -62266,7 +62266,7 @@
       </c>
       <c r="D213" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E213" s="4" t="inlineStr">
@@ -63420,7 +63420,7 @@
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>Bridg</t>
+          <t>BRDG</t>
         </is>
       </c>
       <c r="E227" s="4" t="inlineStr">
@@ -64644,7 +64644,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Append-only record from runner.py (data/raw_quotes.jsonl). Blue = observed values read from each site's UI. Times are UTC with milliseconds. 'Value read at' is when the compared value was read — all sites in a run read at the same moment (snapshot barrier); Δ read = |value read − Bridg's value read| in that run.</t>
+          <t>Append-only record from runner.py (data/raw_quotes.jsonl). Blue = observed values read from each site's UI. Times are UTC with milliseconds. 'Value read at' is when the compared value was read — all sites in a run read at the same moment (snapshot barrier); Δ read = |value read − BRDG's value read| in that run.</t>
         </is>
       </c>
     </row>
@@ -64707,7 +64707,7 @@
       </c>
       <c r="D2" s="23" t="inlineStr">
         <is>
-          <t>ETH→SOL, BSC→SOL, Base→SOL: −19.9 to −20.0 bps in every sample after adding back Bridg's 5 bps. Verified via Bridg's API (indicative quotes, 14:45:35 UTC, saved in data/api/): for a recipient that already holds USDC, Bridg prices Relay at 99.945676 — identical to relay.link. For a fresh Solana address, Relay's 'destination fill gas' rises from 0.004 to 0.205 USDC (+20.1 bps): the cost of creating the recipient's USDC token account. Bridg's no-wallet page prices that case; relay.link's no-wallet page assumes the account exists. Mayan and NEAR Intents shift the same way. SOL→ETH was −25 bps this campaign (Ethereum gas elevated).</t>
+          <t>ETH→SOL, BSC→SOL, Base→SOL: −19.9 to −20.0 bps in every sample after adding back BRDG's 5 bps. Verified via BRDG's API (indicative quotes, 14:45:35 UTC, saved in data/api/): for a recipient that already holds USDC, BRDG prices Relay at 99.945676 — identical to relay.link. For a fresh Solana address, Relay's 'destination fill gas' rises from 0.004 to 0.205 USDC (+20.1 bps): the cost of creating the recipient's USDC token account. BRDG's no-wallet page prices that case; relay.link's no-wallet page assumes the account exists. Mayan and NEAR Intents shift the same way. SOL→ETH was −25 bps this campaign (Ethereum gas elevated).</t>
         </is>
       </c>
     </row>
@@ -64727,7 +64727,7 @@
       </c>
       <c r="D3" s="23" t="inlineStr">
         <is>
-          <t>LI.FI: 15–96 bps below jumper.exchange's Best Return on every route. Bridg's API shows a 'LIFI Fixed Fee' of 0.25 USDC (25 bps) on its LI.FI row that Jumper doesn't charge, plus the ~0.20 new-account cost into Solana — together ~45 bps; the rest is unexplained (likely a different route). SimpleSwap: 48–272 bps below simpleswap.io's default floating 'Best rate'; Bridg's API lists no fee breakdown for it.</t>
+          <t>LI.FI: 15–96 bps below jumper.exchange's Best Return on every route. BRDG's API shows a 'LIFI Fixed Fee' of 0.25 USDC (25 bps) on its LI.FI row that Jumper doesn't charge, plus the ~0.20 new-account cost into Solana — together ~45 bps; the rest is unexplained (likely a different route). SimpleSwap: 48–272 bps below simpleswap.io's default floating 'Best rate'; BRDG's API lists no fee breakdown for it.</t>
         </is>
       </c>
     </row>
@@ -64747,7 +64747,7 @@
       </c>
       <c r="D4" s="23" t="inlineStr">
         <is>
-          <t>Bridg's API fee breakdown: Meson = a fixed 'Meson LP fee' of 0.50 USDC; Husher = fixed 0.20 exchange fee + 0.30 delivery fee; Allbridge = fixed 0.10 CCTP service fee. So Bridg shows exactly 99.5/99.9 minus its own fee (99.45025 / 99.85005; 99.75015 on SOL→ETH at the 15 bps tier). When Ethereum gas rose, Meson's own site dropped to 98.56 on SOL→ETH while Bridg still showed 99.75 (+134 bps). Husher's own site charges 0.35% (not 0.20), so it's 15–25 bps lower than Bridg's row. Allbridge matches because its site also shows a flat 99.90.</t>
+          <t>BRDG's API fee breakdown: Meson = a fixed 'Meson LP fee' of 0.50 USDC; Husher = fixed 0.20 exchange fee + 0.30 delivery fee; Allbridge = fixed 0.10 CCTP service fee. So BRDG shows exactly 99.5/99.9 minus its own fee (99.45025 / 99.85005; 99.75015 on SOL→ETH at the 15 bps tier). When Ethereum gas rose, Meson's own site dropped to 98.56 on SOL→ETH while BRDG still showed 99.75 (+134 bps). Husher's own site charges 0.35% (not 0.20), so it's 15–25 bps lower than BRDG's row. Allbridge matches because its site also shows a flat 99.90.</t>
         </is>
       </c>
     </row>
@@ -64762,12 +64762,12 @@
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>Bridg lists venues whose own site can't quote these routes</t>
+          <t>BRDG lists venues whose own site can't quote these routes</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Rhino.fi (Bridg's best price on SOL→BSC) — retail app shut down Aug 2026. Eco — its portal has no Solana or BNB Chain, yet Bridg lists Eco on SOL↔ETH/Base. NEAR Intents — public app moved behind a login.</t>
+          <t>Rhino.fi (BRDG's best price on SOL→BSC) — retail app shut down Aug 2026. Eco — its portal has no Solana or BNB Chain, yet BRDG lists Eco on SOL↔ETH/Base. NEAR Intents — public app moved behind a login.</t>
         </is>
       </c>
     </row>
@@ -64782,12 +64782,12 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>Across missing from Bridg on 4 of 6 routes</t>
+          <t>Across missing from BRDG on 4 of 6 routes</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Not listed on ETH→SOL, BSC→SOL, Base→SOL or SOL→BSC although across.to quotes 99.98–99.99. Where listed (SOL→ETH, SOL→Base) it matches exactly net of Bridg's fee and is Bridg's best price.</t>
+          <t>Not listed on ETH→SOL, BSC→SOL, Base→SOL or SOL→BSC although across.to quotes 99.98–99.99. Where listed (SOL→ETH, SOL→Base) it matches exactly net of BRDG's fee and is BRDG's best price.</t>
         </is>
       </c>
     </row>
@@ -64802,12 +64802,12 @@
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>Competitor platforms: Bridg beats OpenSea; the rest can't be quoted</t>
+          <t>Competitor platforms: BRDG beats OpenSea; the rest can't be quoted</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>OpenSea swap (Relay; LI.FI on SOL→Base; 0% OpenSea fee promo) pays 89 bps less than Bridg's best on SOL→ETH, ~10 bps less on ETH→SOL and Base→SOL, ~1 bp less on SOL→Base; no BNB Chain. Signed in (by the user) and re-checked: Axiom has a cross-chain Convert, but the amount is capped at the wallet balance, so 100 USDC can't be priced unfunded (deposit fees shown only at its $2–3 minimum). GMGN's Convert needs 2FA plus a 3-hour lock; its deposits are Solana-only. Pump.fun's web deposit is Solana-only. FOMO pools deposits from 7 chains into one USD balance with no quote.</t>
+          <t>OpenSea swap (Relay; LI.FI on SOL→Base; 0% OpenSea fee promo) pays 89 bps less than BRDG's best on SOL→ETH, ~10 bps less on ETH→SOL and Base→SOL, ~1 bp less on SOL→Base; no BNB Chain. Signed in (by the user) and re-checked: Axiom has a cross-chain Convert, but the amount is capped at the wallet balance, so 100 USDC can't be priced unfunded (deposit fees shown only at its $2–3 minimum). GMGN's Convert needs 2FA plus a 3-hour lock; its deposits are Solana-only. Pump.fun's web deposit is Solana-only. FOMO pools deposits from 7 chains into one USD balance with no quote.</t>
         </is>
       </c>
     </row>
@@ -64842,12 +64842,12 @@
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>CCTP gap is Portal hiding a fee, not a Bridg error</t>
+          <t>CCTP gap is Portal hiding a fee, not a BRDG error</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Circle's own bridge has no Solana, so CCTP is read from Portal (Wormhole), which hides its relayer fee until a wallet connects. Bridg's API itemises it: 'Circle Forwarding Service fee and destination gas' = 0.16 USDC on ETH→SOL, which is the −14 to −15 bps gap into Solana. On SOL→ETH (−332 bps this campaign) the same line carries Ethereum destination gas, which was elevated.</t>
+          <t>Circle's own bridge has no Solana, so CCTP is read from Portal (Wormhole), which hides its relayer fee until a wallet connects. BRDG's API itemises it: 'Circle Forwarding Service fee and destination gas' = 0.16 USDC on ETH→SOL, which is the −14 to −15 bps gap into Solana. On SOL→ETH (−332 bps this campaign) the same line carries Ethereum destination gas, which was elevated.</t>
         </is>
       </c>
     </row>
@@ -64862,12 +64862,12 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>Bridg's fee isn't applied to every venue; deBridge's fixed fee jumps around</t>
+          <t>BRDG's fee isn't applied to every venue; deBridge's fixed fee jumps around</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>deBridge, Symbiosis and Mayan (ETH→SOL) match their own sites before adding back Bridg's 5 bps — Bridg appears not to take its fee on those rows. deBridge's own site adds a fixed fee on top of the input that changed a lot between loads (it's compared as out − fee), so some deBridge gaps swing widely.</t>
+          <t>deBridge, Symbiosis and Mayan (ETH→SOL) match their own sites before adding back BRDG's 5 bps — BRDG appears not to take its fee on those rows. deBridge's own site adds a fixed fee on top of the input that changed a lot between loads (it's compared as out − fee), so some deBridge gaps swing widely.</t>
         </is>
       </c>
     </row>
@@ -64887,7 +64887,7 @@
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Across where listed (0.0), Allbridge Core (0.0), Skip Go (+1.2 to +1.6; volatile on SOL→ETH), Mayan on most routes, and Relay on SOL→BSC/SOL→Base match their own sites net of Bridg's fee.</t>
+          <t>Across where listed (0.0), Allbridge Core (0.0), Skip Go (+1.2 to +1.6; volatile on SOL→ETH), Mayan on most routes, and Relay on SOL→BSC/SOL→Base match their own sites net of BRDG's fee.</t>
         </is>
       </c>
     </row>
@@ -64990,7 +64990,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bridg Competitive Benchmark — one-pager</t>
+          <t>BRDG Competitive Benchmark — one-pager</t>
         </is>
       </c>
     </row>
@@ -65358,7 +65358,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Method: fresh Playwright browser per site, no wallet; 100 typed into all pages at one barrier; quotes within ~1.5 s of Bridg's. Evidence: screenshots + SHA-256 in Receipts. Dashboard: see repo README.</t>
+          <t>Method: fresh Playwright browser per site, no wallet; 100 typed into all pages at one barrier; quotes within ~1.5 s of BRDG's. Evidence: screenshots + SHA-256 in Receipts. Dashboard: see repo README.</t>
         </is>
       </c>
     </row>

</xml_diff>